<commit_message>
Actualización automática del sistema Lottery Loop
</commit_message>
<xml_diff>
--- a/data/sugerencias_historico.xlsx
+++ b/data/sugerencias_historico.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H127"/>
+  <dimension ref="A1:H139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2.2494</v>
+        <v>2.0645</v>
       </c>
       <c r="D2" t="n">
         <v>116</v>
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.2229</v>
+        <v>2.0468</v>
       </c>
       <c r="D3" t="n">
         <v>103</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2.1523</v>
+        <v>1.987</v>
       </c>
       <c r="D4" t="n">
         <v>121</v>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.6975</v>
+        <v>1.5728</v>
       </c>
       <c r="D5" t="n">
         <v>115</v>
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.8014</v>
+        <v>1.6693</v>
       </c>
       <c r="D6" t="n">
         <v>96</v>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.6775</v>
+        <v>1.5708</v>
       </c>
       <c r="D7" t="n">
         <v>101</v>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2.455</v>
+        <v>2.2494</v>
       </c>
       <c r="D8" t="n">
         <v>116</v>
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2.4189</v>
+        <v>2.2229</v>
       </c>
       <c r="D9" t="n">
         <v>103</v>
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2.3362</v>
+        <v>2.1523</v>
       </c>
       <c r="D10" t="n">
         <v>121</v>
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1.8362</v>
+        <v>1.6975</v>
       </c>
       <c r="D11" t="n">
         <v>115</v>
@@ -826,14 +826,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[10, 12, 25, 26, 29]</t>
+          <t>[5, 12, 16, 26, 37]</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.9843</v>
+        <v>1.8014</v>
       </c>
       <c r="D12" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -856,14 +856,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[5, 12, 16, 26, 37]</t>
+          <t>[10, 11, 25, 26, 29]</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.9484</v>
+        <v>1.6775</v>
       </c>
       <c r="D13" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2.6835</v>
+        <v>2.2494</v>
       </c>
       <c r="D14" t="n">
         <v>116</v>
@@ -926,7 +926,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.6367</v>
+        <v>2.2229</v>
       </c>
       <c r="D15" t="n">
         <v>103</v>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2.5406</v>
+        <v>2.1523</v>
       </c>
       <c r="D16" t="n">
         <v>121</v>
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.9904</v>
+        <v>1.6975</v>
       </c>
       <c r="D17" t="n">
         <v>115</v>
@@ -1030,14 +1030,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>[10, 12, 25, 26, 29]</t>
+          <t>[5, 12, 16, 26, 37]</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2.1415</v>
+        <v>1.8014</v>
       </c>
       <c r="D18" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1060,14 +1060,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[5, 12, 16, 26, 37]</t>
+          <t>[10, 11, 25, 26, 29]</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2.1117</v>
+        <v>1.6775</v>
       </c>
       <c r="D19" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2.6835</v>
+        <v>2.455</v>
       </c>
       <c r="D20" t="n">
         <v>116</v>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2.6367</v>
+        <v>2.4189</v>
       </c>
       <c r="D21" t="n">
         <v>103</v>
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2.5406</v>
+        <v>2.3362</v>
       </c>
       <c r="D22" t="n">
         <v>121</v>
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.9904</v>
+        <v>1.8362</v>
       </c>
       <c r="D23" t="n">
         <v>115</v>
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2.1415</v>
+        <v>1.9843</v>
       </c>
       <c r="D24" t="n">
         <v>102</v>
@@ -1268,7 +1268,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2.1117</v>
+        <v>1.9484</v>
       </c>
       <c r="D25" t="n">
         <v>96</v>
@@ -4753,6 +4753,414 @@
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>BALOTO</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>[11, 17, 24, 26, 38]</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>2.6835</v>
+      </c>
+      <c r="D128" t="n">
+        <v>116</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G128" t="n">
+        <v>3</v>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>SuperBalota</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>BALOTO</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>[10, 14, 22, 28, 29]</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>2.6367</v>
+      </c>
+      <c r="D129" t="n">
+        <v>103</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G129" t="n">
+        <v>15</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>SuperBalota</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>REVANCHA</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>[15, 18, 22, 28, 38]</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>2.5406</v>
+      </c>
+      <c r="D130" t="n">
+        <v>121</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G130" t="n">
+        <v>13</v>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>SuperBalota</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>REVANCHA</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>[8, 9, 22, 37, 39]</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>1.9904</v>
+      </c>
+      <c r="D131" t="n">
+        <v>115</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G131" t="n">
+        <v>10</v>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>SuperBalota</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>MILOTO</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>[10, 12, 25, 26, 29]</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>2.1415</v>
+      </c>
+      <c r="D132" t="n">
+        <v>102</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>MILOTO</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>[5, 12, 16, 26, 37]</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>2.1117</v>
+      </c>
+      <c r="D133" t="n">
+        <v>96</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>BALOTO</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>[11, 17, 24, 26, 38]</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>2.6835</v>
+      </c>
+      <c r="D134" t="n">
+        <v>116</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G134" t="n">
+        <v>3</v>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>SuperBalota</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>BALOTO</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>[10, 14, 22, 28, 29]</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>2.6367</v>
+      </c>
+      <c r="D135" t="n">
+        <v>103</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G135" t="n">
+        <v>15</v>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>SuperBalota</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>REVANCHA</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>[15, 18, 22, 28, 38]</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>2.5406</v>
+      </c>
+      <c r="D136" t="n">
+        <v>121</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G136" t="n">
+        <v>13</v>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>SuperBalota</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>REVANCHA</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>[8, 9, 22, 37, 39]</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>1.9904</v>
+      </c>
+      <c r="D137" t="n">
+        <v>115</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G137" t="n">
+        <v>10</v>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>SuperBalota</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>MILOTO</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>[10, 12, 25, 26, 29]</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>2.1415</v>
+      </c>
+      <c r="D138" t="n">
+        <v>102</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>MILOTO</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>[5, 12, 16, 26, 37]</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>2.1117</v>
+      </c>
+      <c r="D139" t="n">
+        <v>96</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LOOP-MULTI</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>